<commit_message>
Update Nellie Von Solms title to Miss in UserDetails.xlsx
</commit_message>
<xml_diff>
--- a/users/UserDetails.xlsx
+++ b/users/UserDetails.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apps\AgendaBuilder\users\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B009A54-D65C-47E8-94DB-2D507ED1A7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590701E9-35B4-455D-837A-EE9325417D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5FEAAE74-E41F-4055-98C2-F960B403D25B}"/>
+    <workbookView xWindow="1536" yWindow="1344" windowWidth="17280" windowHeight="10896" xr2:uid="{5FEAAE74-E41F-4055-98C2-F960B403D25B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="99">
   <si>
     <t>Surname</t>
   </si>
@@ -333,6 +333,9 @@
   </si>
   <si>
     <t>15</t>
+  </si>
+  <si>
+    <t>Miss</t>
   </si>
 </sst>
 </file>
@@ -416,9 +419,6 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -436,6 +436,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -775,437 +778,437 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6" style="3" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="3"/>
+    <col min="1" max="1" width="6" style="2" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="4" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="4" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="4" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="4" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="5" t="s">
+      <c r="F16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="5" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>